<commit_message>
feat(excel): tambahkan kolom Tipe Simbol SLD, Dari GI & Ke GI di Jalur_Transmisi dan Gardu_Induk
</commit_message>
<xml_diff>
--- a/peta-kerawanan/public/template_kerawanan_subsistem_suralaya_cilegon.xlsx
+++ b/peta-kerawanan/public/template_kerawanan_subsistem_suralaya_cilegon.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V24"/>
+  <dimension ref="A1:Y21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,57 +416,66 @@
         <v>Tipe Saluran</v>
       </c>
       <c r="E1" t="str">
+        <v>Tipe Simbol SLD</v>
+      </c>
+      <c r="F1" t="str">
         <v>Dari GI</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
+        <v>Tipe Simbol Dari GI</v>
+      </c>
+      <c r="H1" t="str">
         <v>Tier Dari GI</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Ke GI</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
+        <v>Tipe Simbol Ke GI</v>
+      </c>
+      <c r="K1" t="str">
         <v>Tier Ke GI</v>
       </c>
-      <c r="I1" t="str">
+      <c r="L1" t="str">
         <v>Tegangan</v>
       </c>
-      <c r="J1" t="str">
+      <c r="M1" t="str">
         <v>Jumlah Sirkit</v>
       </c>
-      <c r="K1" t="str">
+      <c r="N1" t="str">
         <v>No Sirkit</v>
       </c>
-      <c r="L1" t="str">
+      <c r="O1" t="str">
         <v>Status Operasi</v>
       </c>
-      <c r="M1" t="str">
+      <c r="P1" t="str">
         <v>Tingkat Kerawanan</v>
       </c>
-      <c r="N1" t="str">
+      <c r="Q1" t="str">
         <v>Pembebanan Sirkit 1 (%)</v>
       </c>
-      <c r="O1" t="str">
+      <c r="R1" t="str">
         <v>Pembebanan Sirkit 2 (%)</v>
       </c>
-      <c r="P1" t="str">
+      <c r="S1" t="str">
         <v>Panjang Saluran (km)</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="T1" t="str">
         <v>Koridor / Wilayah</v>
       </c>
-      <c r="R1" t="str">
+      <c r="U1" t="str">
         <v>UIT</v>
       </c>
-      <c r="S1" t="str">
+      <c r="V1" t="str">
         <v>Kondisi / Permasalahan</v>
       </c>
-      <c r="T1" t="str">
+      <c r="W1" t="str">
         <v>Dampak</v>
       </c>
-      <c r="U1" t="str">
+      <c r="X1" t="str">
         <v>Mitigasi</v>
       </c>
-      <c r="V1" t="str">
+      <c r="Y1" t="str">
         <v>Usulan / Solusi</v>
       </c>
     </row>
@@ -484,61 +493,70 @@
         <v>Bay IBT</v>
       </c>
       <c r="E2" t="str">
+        <v>IBT</v>
+      </c>
+      <c r="F2" t="str">
         <v>Suralaya Baru</v>
       </c>
-      <c r="F2">
+      <c r="G2" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H2">
         <v>0</v>
       </c>
-      <c r="G2" t="str">
+      <c r="I2" t="str">
         <v>SRLYA</v>
       </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2" t="str">
         <v>500/150 kV</v>
       </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2" t="str">
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M2" t="str">
+      <c r="P2" t="str">
         <v>Sangat Rawan</v>
       </c>
-      <c r="N2">
+      <c r="Q2">
         <v>88</v>
       </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2">
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2">
         <v>0.5</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="T2" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R2" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S2" t="str">
+      <c r="U2" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="V2" t="str">
         <v>Pembebanan IBT–1,2 Suralaya tidak memenuhi kriteria N–1 saat PLTU Suralaya unit–3 tidak beroperasi dan IBT–4 Cilegon masuk sub sistem Cilegon.</v>
       </c>
-      <c r="T2" t="str" xml:space="preserve">
+      <c r="W2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Pemeliharaan IBT sulit dilakukan.
 2. Pertumbuhan beban menjadi terhambat.
 3. Terjadi pemadaman apabila trip salah satu IBT di Suralaya.</v>
       </c>
-      <c r="U2" t="str" xml:space="preserve">
+      <c r="X2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW.
 2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan total target sebesar 137 MW.
 3. Pemeliharaan IBT saat beban rendah.</v>
       </c>
-      <c r="V2" t="str" xml:space="preserve">
+      <c r="Y2" t="str" xml:space="preserve">
         <v xml:space="preserve">Jangka Pendek :
 Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD di Tahun 2025.</v>
       </c>
@@ -557,59 +575,68 @@
         <v>Bay IBT</v>
       </c>
       <c r="E3" t="str">
+        <v>IBT</v>
+      </c>
+      <c r="F3" t="str">
         <v>Suralaya</v>
       </c>
-      <c r="F3">
+      <c r="G3" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H3">
         <v>0</v>
       </c>
-      <c r="G3" t="str">
+      <c r="I3" t="str">
         <v>SRLYA</v>
       </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3" t="str">
         <v>500/150 kV</v>
       </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3" t="str">
+      <c r="M3">
+        <v>1</v>
+      </c>
+      <c r="N3">
+        <v>1</v>
+      </c>
+      <c r="O3" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M3" t="str">
+      <c r="P3" t="str">
         <v>Sangat Rawan</v>
       </c>
-      <c r="N3">
+      <c r="Q3">
         <v>84</v>
       </c>
-      <c r="O3" t="str">
-        <v/>
-      </c>
-      <c r="P3">
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3">
         <v>0.5</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="T3" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R3" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S3" t="str">
+      <c r="U3" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="V3" t="str">
         <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #1,2 Suralaya 250 MVA sedangkan IBT #4 Cilegon 500 MVA).</v>
       </c>
-      <c r="T3" t="str" xml:space="preserve">
+      <c r="W3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Ketidakseimbangan beban antara IBT Suralaya dan IBT Cilegon.
 2. Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
       </c>
-      <c r="U3" t="str" xml:space="preserve">
+      <c r="X3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya.
 2. Pemeliharaan IBT saat beban rendah.</v>
       </c>
-      <c r="V3" t="str" xml:space="preserve">
+      <c r="Y3" t="str" xml:space="preserve">
         <v xml:space="preserve">Jangka Pendek :
 Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD di Tahun 2026.</v>
       </c>
@@ -628,57 +655,66 @@
         <v>Bay IBT</v>
       </c>
       <c r="E4" t="str">
+        <v>IBT</v>
+      </c>
+      <c r="F4" t="str">
         <v>Cilegon Baru</v>
       </c>
-      <c r="F4">
+      <c r="G4" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H4">
         <v>0</v>
       </c>
-      <c r="G4" t="str">
+      <c r="I4" t="str">
         <v>CLBRU</v>
       </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4" t="str">
         <v>500/150 kV</v>
       </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4" t="str">
+      <c r="M4">
+        <v>1</v>
+      </c>
+      <c r="N4">
+        <v>1</v>
+      </c>
+      <c r="O4" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M4" t="str">
+      <c r="P4" t="str">
         <v>Sangat Rawan</v>
       </c>
-      <c r="N4">
+      <c r="Q4">
         <v>76</v>
       </c>
-      <c r="O4" t="str">
-        <v/>
-      </c>
-      <c r="P4">
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4">
         <v>0.5</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="T4" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R4" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S4" t="str">
+      <c r="U4" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="V4" t="str">
         <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama.</v>
       </c>
-      <c r="T4" t="str">
+      <c r="W4" t="str">
         <v>Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
       </c>
-      <c r="U4" t="str">
+      <c r="X4" t="str">
         <v>Optimalisasi transfer trip dan defense scheme antar GI.</v>
       </c>
-      <c r="V4" t="str" xml:space="preserve">
+      <c r="Y4" t="str" xml:space="preserve">
         <v xml:space="preserve">Jangka Pendek :
 Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA.</v>
       </c>
@@ -697,57 +733,66 @@
         <v>Bay Generator</v>
       </c>
       <c r="E5" t="str">
+        <v>Trafo Generator</v>
+      </c>
+      <c r="F5" t="str">
         <v>Unit 3</v>
       </c>
-      <c r="F5">
+      <c r="G5" t="str">
+        <v>Pembangkit</v>
+      </c>
+      <c r="H5">
         <v>0</v>
       </c>
-      <c r="G5" t="str">
+      <c r="I5" t="str">
         <v>SRLYA</v>
       </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5" t="str">
         <v>500 kV</v>
       </c>
-      <c r="J5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5" t="str">
+      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="N5">
+        <v>1</v>
+      </c>
+      <c r="O5" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M5" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N5">
+      <c r="P5" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q5">
         <v>60</v>
       </c>
-      <c r="O5" t="str">
-        <v/>
-      </c>
-      <c r="P5">
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5">
         <v>0.2</v>
       </c>
-      <c r="Q5" t="str">
+      <c r="T5" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R5" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S5" t="str">
+      <c r="U5" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="V5" t="str">
         <v>Evakuasi daya PLTU Suralaya Unit 3 (1. Pembangkit, 2. Trafo Step-Up, 3. CB).</v>
       </c>
-      <c r="T5" t="str">
-        <v/>
-      </c>
-      <c r="U5" t="str">
-        <v/>
-      </c>
-      <c r="V5" t="str">
+      <c r="W5" t="str">
+        <v/>
+      </c>
+      <c r="X5" t="str">
+        <v/>
+      </c>
+      <c r="Y5" t="str">
         <v/>
       </c>
     </row>
@@ -759,63 +804,72 @@
         <v/>
       </c>
       <c r="C6" t="str">
-        <v>SUTT 150 kV SRLYA - SLRDA</v>
+        <v>Suralaya - Salira Indah (Sirkit 1)</v>
       </c>
       <c r="D6" t="str">
         <v>PHT</v>
       </c>
       <c r="E6" t="str">
+        <v>PHT</v>
+      </c>
+      <c r="F6" t="str">
         <v>SRLYA</v>
       </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
       <c r="G6" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6" t="str">
         <v>SLRDA</v>
       </c>
-      <c r="H6">
+      <c r="J6" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K6">
         <v>2</v>
       </c>
-      <c r="I6" t="str">
+      <c r="L6" t="str">
         <v>150 kV</v>
       </c>
-      <c r="J6">
-        <v>1</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="L6" t="str">
+      <c r="M6">
+        <v>2</v>
+      </c>
+      <c r="N6">
+        <v>1</v>
+      </c>
+      <c r="O6" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M6" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N6">
-        <v>54</v>
-      </c>
-      <c r="O6" t="str">
-        <v/>
-      </c>
-      <c r="P6">
-        <v>14.2</v>
-      </c>
-      <c r="Q6" t="str">
+      <c r="P6" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q6">
+        <v>52</v>
+      </c>
+      <c r="R6">
+        <v>48</v>
+      </c>
+      <c r="S6">
+        <v>12.5</v>
+      </c>
+      <c r="T6" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R6" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S6" t="str">
-        <v/>
-      </c>
-      <c r="T6" t="str">
-        <v/>
-      </c>
       <c r="U6" t="str">
-        <v/>
+        <v>JBB</v>
       </c>
       <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
+        <v/>
+      </c>
+      <c r="X6" t="str">
+        <v/>
+      </c>
+      <c r="Y6" t="str">
         <v/>
       </c>
     </row>
@@ -827,63 +881,72 @@
         <v/>
       </c>
       <c r="C7" t="str">
-        <v>SUTT 150 kV SRLYA - PENDO</v>
+        <v>Suralaya - Salira Indah (Sirkit 2)</v>
       </c>
       <c r="D7" t="str">
         <v>PHT</v>
       </c>
       <c r="E7" t="str">
+        <v>PHT</v>
+      </c>
+      <c r="F7" t="str">
         <v>SRLYA</v>
       </c>
-      <c r="F7">
-        <v>1</v>
-      </c>
       <c r="G7" t="str">
-        <v>PENDO</v>
+        <v>Busbar</v>
       </c>
       <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" t="str">
+        <v>SLRDA</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K7">
         <v>2</v>
       </c>
-      <c r="I7" t="str">
+      <c r="L7" t="str">
         <v>150 kV</v>
       </c>
-      <c r="J7">
-        <v>1</v>
-      </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="L7" t="str">
+      <c r="M7">
+        <v>2</v>
+      </c>
+      <c r="N7">
+        <v>2</v>
+      </c>
+      <c r="O7" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M7" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N7">
+      <c r="P7" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q7">
+        <v>52</v>
+      </c>
+      <c r="R7">
         <v>48</v>
       </c>
-      <c r="O7" t="str">
-        <v/>
-      </c>
-      <c r="P7">
-        <v>12.8</v>
-      </c>
-      <c r="Q7" t="str">
+      <c r="S7">
+        <v>12.5</v>
+      </c>
+      <c r="T7" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R7" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S7" t="str">
-        <v/>
-      </c>
-      <c r="T7" t="str">
-        <v/>
-      </c>
       <c r="U7" t="str">
-        <v/>
+        <v>JBB</v>
       </c>
       <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v/>
+      </c>
+      <c r="X7" t="str">
+        <v/>
+      </c>
+      <c r="Y7" t="str">
         <v/>
       </c>
     </row>
@@ -895,67 +958,76 @@
         <v/>
       </c>
       <c r="C8" t="str">
-        <v>SUTT 150 kV Tie Line SLRDA - PENDO</v>
+        <v>Salira Indah - Pendo</v>
       </c>
       <c r="D8" t="str">
         <v>PHT</v>
       </c>
       <c r="E8" t="str">
+        <v>PHT</v>
+      </c>
+      <c r="F8" t="str">
         <v>SLRDA</v>
       </c>
-      <c r="F8">
-        <v>2</v>
-      </c>
       <c r="G8" t="str">
-        <v>PENDO</v>
+        <v>Busbar</v>
       </c>
       <c r="H8">
         <v>2</v>
       </c>
       <c r="I8" t="str">
+        <v>PENDO</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K8">
+        <v>2</v>
+      </c>
+      <c r="L8" t="str">
         <v>150 kV</v>
       </c>
-      <c r="J8">
-        <v>1</v>
-      </c>
-      <c r="K8">
-        <v>1</v>
-      </c>
-      <c r="L8" t="str">
+      <c r="M8">
+        <v>1</v>
+      </c>
+      <c r="N8">
+        <v>1</v>
+      </c>
+      <c r="O8" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M8" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N8">
-        <v>32</v>
-      </c>
-      <c r="O8" t="str">
-        <v/>
-      </c>
-      <c r="P8">
-        <v>6.4</v>
-      </c>
-      <c r="Q8" t="str">
+      <c r="P8" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q8">
+        <v>45</v>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8">
+        <v>8.4</v>
+      </c>
+      <c r="T8" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R8" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S8" t="str">
-        <v>Interkoneksi antar bay busbar SLRDA dan PENDO.</v>
-      </c>
-      <c r="T8" t="str">
-        <v/>
-      </c>
       <c r="U8" t="str">
-        <v/>
+        <v>JBB</v>
       </c>
       <c r="V8" t="str">
         <v/>
       </c>
-    </row>
-    <row r="9" xml:space="preserve">
+      <c r="W8" t="str">
+        <v/>
+      </c>
+      <c r="X8" t="str">
+        <v/>
+      </c>
+      <c r="Y8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9">
         <v>8</v>
       </c>
@@ -963,70 +1035,76 @@
         <v>3</v>
       </c>
       <c r="C9" t="str">
-        <v>SUTT 150 kV SRLYA - PENI (Ruas Suralaya - Peni)</v>
+        <v>Suralaya - Chandra Asri (PENI)</v>
       </c>
       <c r="D9" t="str">
         <v>PHT</v>
       </c>
       <c r="E9" t="str">
+        <v>PHT</v>
+      </c>
+      <c r="F9" t="str">
         <v>SRLYA</v>
       </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
       <c r="G9" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9" t="str">
         <v>PENI</v>
       </c>
-      <c r="H9">
+      <c r="J9" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K9">
         <v>2</v>
       </c>
-      <c r="I9" t="str">
+      <c r="L9" t="str">
         <v>150 kV</v>
       </c>
-      <c r="J9">
-        <v>1</v>
-      </c>
-      <c r="K9">
-        <v>1</v>
-      </c>
-      <c r="L9" t="str">
+      <c r="M9">
+        <v>1</v>
+      </c>
+      <c r="N9">
+        <v>1</v>
+      </c>
+      <c r="O9" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M9" t="str">
+      <c r="P9" t="str">
         <v>N-1</v>
       </c>
-      <c r="N9">
-        <v>74</v>
-      </c>
-      <c r="O9" t="str">
-        <v/>
-      </c>
-      <c r="P9">
-        <v>18.5</v>
-      </c>
-      <c r="Q9" t="str">
+      <c r="Q9">
+        <v>78</v>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9">
+        <v>15.2</v>
+      </c>
+      <c r="T9" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R9" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S9" t="str">
-        <v>Ruas Penghantar Suralaya–MCCI–Cilegon dan Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
-      </c>
-      <c r="T9" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Pemeliharaan Penghantar menjadi sulit dilakukan.
-2. Terjadi pemadaman apabila terdapat gangguan N–1–1.</v>
-      </c>
-      <c r="U9" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Pemeliharaan Penghantar menyesuaikan jadwal dari KTT.
-2. Pengaturan konfigurasi jaringan saat pemeliharaan.</v>
-      </c>
-      <c r="V9" t="str" xml:space="preserve">
-        <v xml:space="preserve">Jangka Menengah :
-Usulan Double phi pada ruas Suralaya s.d Cilegon Lama. Diusulkan COD Tahun 2030.</v>
-      </c>
-    </row>
-    <row r="10" xml:space="preserve">
+      <c r="U9" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="V9" t="str">
+        <v>Ruas Penghantar Suralaya-PENI masih single phi.</v>
+      </c>
+      <c r="W9" t="str">
+        <v>Pemadaman apabila trip saat pemeliharaan KTT.</v>
+      </c>
+      <c r="X9" t="str">
+        <v>Penyesuaian jadwal pemeliharaan.</v>
+      </c>
+      <c r="Y9" t="str">
+        <v>Double phi COD 2030.</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1034,65 +1112,73 @@
         <v>3</v>
       </c>
       <c r="C10" t="str">
-        <v>SUTT 150 kV SRLYA - MCCI5 (Ruas Suralaya - MCCI)</v>
+        <v>Suralaya - MCCI</v>
       </c>
       <c r="D10" t="str">
         <v>PHT</v>
       </c>
       <c r="E10" t="str">
+        <v>PHT</v>
+      </c>
+      <c r="F10" t="str">
         <v>SRLYA</v>
       </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
       <c r="G10" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10" t="str">
         <v>MCCI5</v>
       </c>
-      <c r="H10">
+      <c r="J10" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K10">
         <v>2</v>
       </c>
-      <c r="I10" t="str">
+      <c r="L10" t="str">
         <v>150 kV</v>
       </c>
-      <c r="J10">
-        <v>1</v>
-      </c>
-      <c r="K10">
-        <v>1</v>
-      </c>
-      <c r="L10" t="str">
+      <c r="M10">
+        <v>1</v>
+      </c>
+      <c r="N10">
+        <v>1</v>
+      </c>
+      <c r="O10" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M10" t="str">
+      <c r="P10" t="str">
         <v>N-1</v>
       </c>
-      <c r="N10">
-        <v>71</v>
-      </c>
-      <c r="O10" t="str">
-        <v/>
-      </c>
-      <c r="P10">
-        <v>16.3</v>
-      </c>
-      <c r="Q10" t="str">
+      <c r="Q10">
+        <v>72</v>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10">
+        <v>16.8</v>
+      </c>
+      <c r="T10" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R10" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S10" t="str">
-        <v>Ruas Penghantar Suralaya–MCCI–Cilegon masih single phi.</v>
-      </c>
-      <c r="T10" t="str">
-        <v>Pemadaman apabila terjadi gangguan N-1-1.</v>
-      </c>
       <c r="U10" t="str">
-        <v>Pemeliharaan Penghantar menyesuaikan jadwal dari KTT.</v>
-      </c>
-      <c r="V10" t="str" xml:space="preserve">
-        <v xml:space="preserve">Jangka Menengah :
-Usulan Double phi.</v>
+        <v>JBB</v>
+      </c>
+      <c r="V10" t="str">
+        <v>Ruas Penghantar Suralaya-MCCI-Cilegon masih single phi.</v>
+      </c>
+      <c r="W10" t="str">
+        <v>Pemadaman apabila terjadi trip.</v>
+      </c>
+      <c r="X10" t="str">
+        <v>Penyesuaian jadwal pemeliharaan dari KTT.</v>
+      </c>
+      <c r="Y10" t="str">
+        <v>Usulan double phi ruas Suralaya s.d Cilegon Lama.</v>
       </c>
     </row>
     <row r="11">
@@ -1103,63 +1189,72 @@
         <v/>
       </c>
       <c r="C11" t="str">
-        <v>SUTT 150 kV CLBRU - CLGON Sirkit 1 (2 Line)</v>
+        <v>Cilegon Baru - Cilegon Lama (Sirkit 1)</v>
       </c>
       <c r="D11" t="str">
         <v>PHT</v>
       </c>
       <c r="E11" t="str">
+        <v>PHT</v>
+      </c>
+      <c r="F11" t="str">
         <v>CLBRU</v>
       </c>
-      <c r="F11">
-        <v>1</v>
-      </c>
       <c r="G11" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11" t="str">
         <v>CLGON</v>
       </c>
-      <c r="H11">
+      <c r="J11" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K11">
         <v>2</v>
       </c>
-      <c r="I11" t="str">
+      <c r="L11" t="str">
         <v>150 kV</v>
       </c>
-      <c r="J11">
+      <c r="M11">
         <v>2</v>
       </c>
-      <c r="K11">
-        <v>1</v>
-      </c>
-      <c r="L11" t="str">
+      <c r="N11">
+        <v>1</v>
+      </c>
+      <c r="O11" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M11" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N11">
-        <v>62</v>
-      </c>
-      <c r="O11">
+      <c r="P11" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q11">
+        <v>54</v>
+      </c>
+      <c r="R11">
         <v>50</v>
       </c>
-      <c r="P11">
-        <v>11.2</v>
-      </c>
-      <c r="Q11" t="str">
+      <c r="S11">
+        <v>9.2</v>
+      </c>
+      <c r="T11" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R11" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S11" t="str">
-        <v>Jalur ganda menghubungkan Cilegon Baru dan Cilegon Lama Sirkit 1.</v>
-      </c>
-      <c r="T11" t="str">
-        <v/>
-      </c>
       <c r="U11" t="str">
-        <v/>
+        <v>JBB</v>
       </c>
       <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
+      </c>
+      <c r="X11" t="str">
+        <v/>
+      </c>
+      <c r="Y11" t="str">
         <v/>
       </c>
     </row>
@@ -1171,63 +1266,72 @@
         <v/>
       </c>
       <c r="C12" t="str">
-        <v>SUTT 150 kV CLBRU - CLGON Sirkit 2 (2 Line)</v>
+        <v>Cilegon Baru - Cilegon Lama (Sirkit 2)</v>
       </c>
       <c r="D12" t="str">
         <v>PHT</v>
       </c>
       <c r="E12" t="str">
+        <v>PHT</v>
+      </c>
+      <c r="F12" t="str">
         <v>CLBRU</v>
       </c>
-      <c r="F12">
-        <v>1</v>
-      </c>
       <c r="G12" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H12">
+        <v>1</v>
+      </c>
+      <c r="I12" t="str">
         <v>CLGON</v>
       </c>
-      <c r="H12">
-        <v>2</v>
-      </c>
-      <c r="I12" t="str">
-        <v>150 kV</v>
-      </c>
-      <c r="J12">
-        <v>2</v>
+      <c r="J12" t="str">
+        <v>Busbar</v>
       </c>
       <c r="K12">
         <v>2</v>
       </c>
       <c r="L12" t="str">
+        <v>150 kV</v>
+      </c>
+      <c r="M12">
+        <v>2</v>
+      </c>
+      <c r="N12">
+        <v>2</v>
+      </c>
+      <c r="O12" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M12" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N12">
+      <c r="P12" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q12">
+        <v>54</v>
+      </c>
+      <c r="R12">
         <v>50</v>
       </c>
-      <c r="O12">
-        <v>62</v>
-      </c>
-      <c r="P12">
-        <v>11.2</v>
-      </c>
-      <c r="Q12" t="str">
+      <c r="S12">
+        <v>9.2</v>
+      </c>
+      <c r="T12" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R12" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S12" t="str">
-        <v>Jalur ganda menghubungkan Cilegon Baru dan Cilegon Lama Sirkit 2.</v>
-      </c>
-      <c r="T12" t="str">
-        <v/>
-      </c>
       <c r="U12" t="str">
-        <v/>
+        <v>JBB</v>
       </c>
       <c r="V12" t="str">
+        <v/>
+      </c>
+      <c r="W12" t="str">
+        <v/>
+      </c>
+      <c r="X12" t="str">
+        <v/>
+      </c>
+      <c r="Y12" t="str">
         <v/>
       </c>
     </row>
@@ -1239,64 +1343,73 @@
         <v>3</v>
       </c>
       <c r="C13" t="str">
-        <v>SUTT 150 kV PENI - MTSUI (Ruas Peni - Mitsui)</v>
+        <v>Chandra Asri (PENI) - Mitsui (MTSUI)</v>
       </c>
       <c r="D13" t="str">
         <v>PHT</v>
       </c>
       <c r="E13" t="str">
+        <v>PHT</v>
+      </c>
+      <c r="F13" t="str">
         <v>PENI</v>
       </c>
-      <c r="F13">
+      <c r="G13" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H13">
         <v>2</v>
       </c>
-      <c r="G13" t="str">
+      <c r="I13" t="str">
         <v>MTSUI</v>
       </c>
-      <c r="H13">
+      <c r="J13" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K13">
         <v>3</v>
       </c>
-      <c r="I13" t="str">
+      <c r="L13" t="str">
         <v>150 kV</v>
       </c>
-      <c r="J13">
-        <v>1</v>
-      </c>
-      <c r="K13">
-        <v>1</v>
-      </c>
-      <c r="L13" t="str">
+      <c r="M13">
+        <v>1</v>
+      </c>
+      <c r="N13">
+        <v>1</v>
+      </c>
+      <c r="O13" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M13" t="str">
+      <c r="P13" t="str">
         <v>N-1</v>
       </c>
-      <c r="N13">
-        <v>68</v>
-      </c>
-      <c r="O13" t="str">
-        <v/>
-      </c>
-      <c r="P13">
-        <v>8.7</v>
-      </c>
-      <c r="Q13" t="str">
+      <c r="Q13">
+        <v>65</v>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13">
+        <v>6.8</v>
+      </c>
+      <c r="T13" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R13" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S13" t="str">
-        <v>Ruas Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
-      </c>
-      <c r="T13" t="str">
-        <v>Pemadaman apabila trip saat beban puncak.</v>
-      </c>
       <c r="U13" t="str">
-        <v>Pengaturan operasi terkoordinasi UP2B Banten.</v>
+        <v>JBB</v>
       </c>
       <c r="V13" t="str">
-        <v>Usulan Double phi.</v>
+        <v>Ruas Peni-Mitsui-Cilegon masih single phi.</v>
+      </c>
+      <c r="W13" t="str">
+        <v>Pemadaman apabila trip.</v>
+      </c>
+      <c r="X13" t="str">
+        <v>Jadwal pemeliharaan KTT.</v>
+      </c>
+      <c r="Y13" t="str">
+        <v>Usulan double phi COD 2030.</v>
       </c>
     </row>
     <row r="14">
@@ -1304,67 +1417,76 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="C14" t="str">
-        <v>SUTT 150 kV MCCI5 - CLGON (Ruas MCCI - Cilegon)</v>
+        <v>Mitsui (MTSUI) - Cilegon Lama</v>
       </c>
       <c r="D14" t="str">
         <v>PHT</v>
       </c>
       <c r="E14" t="str">
-        <v>MCCI5</v>
-      </c>
-      <c r="F14">
+        <v>PHT</v>
+      </c>
+      <c r="F14" t="str">
+        <v>MTSUI</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H14">
+        <v>3</v>
+      </c>
+      <c r="I14" t="str">
+        <v>CLGON</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K14">
         <v>2</v>
       </c>
-      <c r="G14" t="str">
-        <v>CLGON</v>
-      </c>
-      <c r="H14">
-        <v>2</v>
-      </c>
-      <c r="I14" t="str">
+      <c r="L14" t="str">
         <v>150 kV</v>
       </c>
-      <c r="J14">
-        <v>1</v>
-      </c>
-      <c r="K14">
-        <v>1</v>
-      </c>
-      <c r="L14" t="str">
+      <c r="M14">
+        <v>1</v>
+      </c>
+      <c r="N14">
+        <v>1</v>
+      </c>
+      <c r="O14" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M14" t="str">
-        <v>N-1</v>
-      </c>
-      <c r="N14">
-        <v>65</v>
-      </c>
-      <c r="O14" t="str">
-        <v/>
-      </c>
-      <c r="P14">
-        <v>9.4</v>
-      </c>
-      <c r="Q14" t="str">
+      <c r="P14" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q14">
+        <v>48</v>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
+      <c r="S14">
+        <v>5.4</v>
+      </c>
+      <c r="T14" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R14" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S14" t="str">
-        <v>Ruas Suralaya–MCCI–Cilegon masih single phi.</v>
-      </c>
-      <c r="T14" t="str">
-        <v>Risiko keandalan suplai pelanggan industri.</v>
-      </c>
       <c r="U14" t="str">
-        <v>Penyesuaian pola operasi jaringan.</v>
+        <v>JBB</v>
       </c>
       <c r="V14" t="str">
-        <v>Usulan Double phi.</v>
+        <v/>
+      </c>
+      <c r="W14" t="str">
+        <v/>
+      </c>
+      <c r="X14" t="str">
+        <v/>
+      </c>
+      <c r="Y14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -1375,63 +1497,72 @@
         <v/>
       </c>
       <c r="C15" t="str">
-        <v>Feeder Trafo SLRDA ke KTT SLFDO-1</v>
+        <v>Feeder Beban KTT SLFDO-1 (78 MVA)</v>
       </c>
       <c r="D15" t="str">
         <v>Feeder Beban</v>
       </c>
       <c r="E15" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="F15" t="str">
         <v>SLRDA</v>
       </c>
-      <c r="F15">
+      <c r="G15" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H15">
         <v>2</v>
       </c>
-      <c r="G15" t="str">
+      <c r="I15" t="str">
         <v>KTT SLFDO-1</v>
       </c>
-      <c r="H15">
+      <c r="J15" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="K15">
         <v>3</v>
       </c>
-      <c r="I15" t="str">
-        <v>150/20 kV</v>
-      </c>
-      <c r="J15">
-        <v>1</v>
-      </c>
-      <c r="K15">
-        <v>1</v>
-      </c>
       <c r="L15" t="str">
+        <v>20 kV</v>
+      </c>
+      <c r="M15">
+        <v>1</v>
+      </c>
+      <c r="N15">
+        <v>1</v>
+      </c>
+      <c r="O15" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M15" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N15">
-        <v>72</v>
-      </c>
-      <c r="O15" t="str">
-        <v/>
-      </c>
-      <c r="P15">
+      <c r="P15" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q15">
+        <v>78</v>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15">
         <v>1.2</v>
       </c>
-      <c r="Q15" t="str">
+      <c r="T15" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R15" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S15" t="str">
-        <v>Suplai konsumen KTT SLFDO-1 Kapasitas 78 MVA.</v>
-      </c>
-      <c r="T15" t="str">
-        <v/>
-      </c>
       <c r="U15" t="str">
-        <v/>
+        <v>JBB</v>
       </c>
       <c r="V15" t="str">
+        <v>Feeder Konsumen Industri KTT SLFDO-1</v>
+      </c>
+      <c r="W15" t="str">
+        <v/>
+      </c>
+      <c r="X15" t="str">
+        <v/>
+      </c>
+      <c r="Y15" t="str">
         <v/>
       </c>
     </row>
@@ -1443,63 +1574,72 @@
         <v/>
       </c>
       <c r="C16" t="str">
-        <v>Feeder Trafo SLRDA ke KTT SLFDO-2</v>
+        <v>Feeder Beban KTT SLFDO-2 (30 MVA)</v>
       </c>
       <c r="D16" t="str">
         <v>Feeder Beban</v>
       </c>
       <c r="E16" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="F16" t="str">
         <v>SLRDA</v>
       </c>
-      <c r="F16">
+      <c r="G16" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H16">
         <v>2</v>
       </c>
-      <c r="G16" t="str">
+      <c r="I16" t="str">
         <v>KTT SLFDO-2</v>
       </c>
-      <c r="H16">
+      <c r="J16" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="K16">
         <v>3</v>
       </c>
-      <c r="I16" t="str">
-        <v>150/20 kV</v>
-      </c>
-      <c r="J16">
-        <v>1</v>
-      </c>
-      <c r="K16">
-        <v>1</v>
-      </c>
       <c r="L16" t="str">
+        <v>20 kV</v>
+      </c>
+      <c r="M16">
+        <v>1</v>
+      </c>
+      <c r="N16">
+        <v>1</v>
+      </c>
+      <c r="O16" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M16" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N16">
-        <v>65</v>
-      </c>
-      <c r="O16" t="str">
-        <v/>
-      </c>
-      <c r="P16">
-        <v>1</v>
-      </c>
-      <c r="Q16" t="str">
+      <c r="P16" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q16">
+        <v>30</v>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
+      <c r="S16">
+        <v>1.2</v>
+      </c>
+      <c r="T16" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R16" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S16" t="str">
-        <v>Suplai konsumen KTT SLFDO-2 Kapasitas 30 MVA.</v>
-      </c>
-      <c r="T16" t="str">
-        <v/>
-      </c>
       <c r="U16" t="str">
-        <v/>
+        <v>JBB</v>
       </c>
       <c r="V16" t="str">
+        <v>Feeder Konsumen Industri KTT SLFDO-2</v>
+      </c>
+      <c r="W16" t="str">
+        <v/>
+      </c>
+      <c r="X16" t="str">
+        <v/>
+      </c>
+      <c r="Y16" t="str">
         <v/>
       </c>
     </row>
@@ -1511,63 +1651,72 @@
         <v/>
       </c>
       <c r="C17" t="str">
-        <v>Feeder Trafo PENDO ke KTT PENDO</v>
+        <v>Feeder Beban KTT PENDO (35 MVA)</v>
       </c>
       <c r="D17" t="str">
         <v>Feeder Beban</v>
       </c>
       <c r="E17" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="F17" t="str">
         <v>PENDO</v>
       </c>
-      <c r="F17">
+      <c r="G17" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H17">
         <v>2</v>
       </c>
-      <c r="G17" t="str">
+      <c r="I17" t="str">
         <v>KTT PENDO</v>
       </c>
-      <c r="H17">
+      <c r="J17" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="K17">
         <v>3</v>
       </c>
-      <c r="I17" t="str">
-        <v>150/20 kV</v>
-      </c>
-      <c r="J17">
-        <v>1</v>
-      </c>
-      <c r="K17">
-        <v>1</v>
-      </c>
       <c r="L17" t="str">
+        <v>20 kV</v>
+      </c>
+      <c r="M17">
+        <v>1</v>
+      </c>
+      <c r="N17">
+        <v>1</v>
+      </c>
+      <c r="O17" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M17" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N17">
-        <v>58</v>
-      </c>
-      <c r="O17" t="str">
-        <v/>
-      </c>
-      <c r="P17">
+      <c r="P17" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q17">
+        <v>35</v>
+      </c>
+      <c r="R17" t="str">
+        <v/>
+      </c>
+      <c r="S17">
         <v>0.8</v>
       </c>
-      <c r="Q17" t="str">
+      <c r="T17" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R17" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S17" t="str">
-        <v>Suplai konsumen KTT PENDO Kapasitas 35 MVA.</v>
-      </c>
-      <c r="T17" t="str">
-        <v/>
-      </c>
       <c r="U17" t="str">
-        <v/>
+        <v>JBB</v>
       </c>
       <c r="V17" t="str">
+        <v>Feeder Konsumen Industri KTT PENDO</v>
+      </c>
+      <c r="W17" t="str">
+        <v/>
+      </c>
+      <c r="X17" t="str">
+        <v/>
+      </c>
+      <c r="Y17" t="str">
         <v/>
       </c>
     </row>
@@ -1576,66 +1725,75 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="C18" t="str">
-        <v>Feeder Trafo PENI ke KTT PENI</v>
+        <v>Feeder Beban KTT PENI (40 MVA)</v>
       </c>
       <c r="D18" t="str">
         <v>Feeder Beban</v>
       </c>
       <c r="E18" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="F18" t="str">
         <v>PENI</v>
       </c>
-      <c r="F18">
+      <c r="G18" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H18">
         <v>2</v>
       </c>
-      <c r="G18" t="str">
+      <c r="I18" t="str">
         <v>KTT PENI</v>
       </c>
-      <c r="H18">
+      <c r="J18" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="K18">
         <v>3</v>
       </c>
-      <c r="I18" t="str">
-        <v>150/20 kV</v>
-      </c>
-      <c r="J18">
-        <v>1</v>
-      </c>
-      <c r="K18">
-        <v>1</v>
-      </c>
       <c r="L18" t="str">
+        <v>20 kV</v>
+      </c>
+      <c r="M18">
+        <v>1</v>
+      </c>
+      <c r="N18">
+        <v>1</v>
+      </c>
+      <c r="O18" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M18" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N18">
-        <v>60</v>
-      </c>
-      <c r="O18" t="str">
-        <v/>
-      </c>
-      <c r="P18">
-        <v>1.1</v>
-      </c>
-      <c r="Q18" t="str">
+      <c r="P18" t="str">
+        <v>N-1</v>
+      </c>
+      <c r="Q18">
+        <v>40</v>
+      </c>
+      <c r="R18" t="str">
+        <v/>
+      </c>
+      <c r="S18">
+        <v>0.5</v>
+      </c>
+      <c r="T18" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R18" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S18" t="str">
-        <v>Suplai konsumen KTT PENI Kapasitas 40 MVA.</v>
-      </c>
-      <c r="T18" t="str">
-        <v/>
-      </c>
       <c r="U18" t="str">
-        <v/>
+        <v>JBB</v>
       </c>
       <c r="V18" t="str">
+        <v>Feeder Konsumen Industri KTT PENI</v>
+      </c>
+      <c r="W18" t="str">
+        <v/>
+      </c>
+      <c r="X18" t="str">
+        <v/>
+      </c>
+      <c r="Y18" t="str">
         <v/>
       </c>
     </row>
@@ -1647,63 +1805,72 @@
         <v/>
       </c>
       <c r="C19" t="str">
-        <v>Feeder Trafo PENI ke KTT LCI (2 Line)</v>
+        <v>Feeder Beban KTT LCI (115 MVA)</v>
       </c>
       <c r="D19" t="str">
         <v>Feeder Beban</v>
       </c>
       <c r="E19" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="F19" t="str">
         <v>PENI</v>
       </c>
-      <c r="F19">
+      <c r="G19" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H19">
         <v>2</v>
       </c>
-      <c r="G19" t="str">
+      <c r="I19" t="str">
         <v>KTT LCI</v>
       </c>
-      <c r="H19">
+      <c r="J19" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="K19">
         <v>3</v>
       </c>
-      <c r="I19" t="str">
-        <v>150/20 kV</v>
-      </c>
-      <c r="J19">
+      <c r="L19" t="str">
+        <v>20 kV</v>
+      </c>
+      <c r="M19">
         <v>2</v>
       </c>
-      <c r="K19">
-        <v>1</v>
-      </c>
-      <c r="L19" t="str">
+      <c r="N19">
+        <v>1</v>
+      </c>
+      <c r="O19" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M19" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N19">
-        <v>64</v>
-      </c>
-      <c r="O19">
-        <v>60</v>
-      </c>
-      <c r="P19">
+      <c r="P19" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q19">
+        <v>58</v>
+      </c>
+      <c r="R19">
+        <v>57</v>
+      </c>
+      <c r="S19">
         <v>1.5</v>
       </c>
-      <c r="Q19" t="str">
+      <c r="T19" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R19" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S19" t="str">
-        <v>Suplai 2 sirkit konsumen KTT LCI Kapasitas 115 MVA.</v>
-      </c>
-      <c r="T19" t="str">
-        <v/>
-      </c>
       <c r="U19" t="str">
-        <v/>
+        <v>JBB</v>
       </c>
       <c r="V19" t="str">
+        <v>Feeder Konsumen Industri KTT LCI</v>
+      </c>
+      <c r="W19" t="str">
+        <v/>
+      </c>
+      <c r="X19" t="str">
+        <v/>
+      </c>
+      <c r="Y19" t="str">
         <v/>
       </c>
     </row>
@@ -1715,63 +1882,72 @@
         <v/>
       </c>
       <c r="C20" t="str">
-        <v>Feeder Trafo MCCI5 ke KTT MCCI</v>
+        <v>Feeder Beban KTT MCCI (40 MVA)</v>
       </c>
       <c r="D20" t="str">
         <v>Feeder Beban</v>
       </c>
       <c r="E20" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="F20" t="str">
         <v>MCCI5</v>
       </c>
-      <c r="F20">
+      <c r="G20" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H20">
         <v>2</v>
       </c>
-      <c r="G20" t="str">
+      <c r="I20" t="str">
         <v>KTT MCCI</v>
       </c>
-      <c r="H20">
+      <c r="J20" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="K20">
         <v>3</v>
       </c>
-      <c r="I20" t="str">
-        <v>150/20 kV</v>
-      </c>
-      <c r="J20">
-        <v>1</v>
-      </c>
-      <c r="K20">
-        <v>1</v>
-      </c>
       <c r="L20" t="str">
+        <v>20 kV</v>
+      </c>
+      <c r="M20">
+        <v>1</v>
+      </c>
+      <c r="N20">
+        <v>1</v>
+      </c>
+      <c r="O20" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M20" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N20">
-        <v>55</v>
-      </c>
-      <c r="O20" t="str">
-        <v/>
-      </c>
-      <c r="P20">
-        <v>0.9</v>
-      </c>
-      <c r="Q20" t="str">
+      <c r="P20" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q20">
+        <v>40</v>
+      </c>
+      <c r="R20" t="str">
+        <v/>
+      </c>
+      <c r="S20">
+        <v>0.6</v>
+      </c>
+      <c r="T20" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R20" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S20" t="str">
-        <v>Suplai konsumen KTT MCCI Kapasitas 40 MVA.</v>
-      </c>
-      <c r="T20" t="str">
-        <v/>
-      </c>
       <c r="U20" t="str">
-        <v/>
+        <v>JBB</v>
       </c>
       <c r="V20" t="str">
+        <v>Feeder Konsumen Industri KTT MCCI</v>
+      </c>
+      <c r="W20" t="str">
+        <v/>
+      </c>
+      <c r="X20" t="str">
+        <v/>
+      </c>
+      <c r="Y20" t="str">
         <v/>
       </c>
     </row>
@@ -1783,273 +1959,78 @@
         <v/>
       </c>
       <c r="C21" t="str">
-        <v>Feeder Trafo MTSUI ke KTT MTSUI</v>
+        <v>Feeder Beban KTT MTSUI (31 MVA)</v>
       </c>
       <c r="D21" t="str">
         <v>Feeder Beban</v>
       </c>
       <c r="E21" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="F21" t="str">
         <v>MTSUI</v>
       </c>
-      <c r="F21">
+      <c r="G21" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H21">
         <v>3</v>
       </c>
-      <c r="G21" t="str">
+      <c r="I21" t="str">
         <v>KTT MTSUI</v>
       </c>
-      <c r="H21">
+      <c r="J21" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="K21">
         <v>4</v>
       </c>
-      <c r="I21" t="str">
-        <v>150/20 kV</v>
-      </c>
-      <c r="J21">
-        <v>1</v>
-      </c>
-      <c r="K21">
-        <v>1</v>
-      </c>
       <c r="L21" t="str">
+        <v>20 kV</v>
+      </c>
+      <c r="M21">
+        <v>1</v>
+      </c>
+      <c r="N21">
+        <v>1</v>
+      </c>
+      <c r="O21" t="str">
         <v>Beroperasi</v>
       </c>
-      <c r="M21" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N21">
-        <v>50</v>
-      </c>
-      <c r="O21" t="str">
-        <v/>
-      </c>
-      <c r="P21">
-        <v>0.7</v>
-      </c>
-      <c r="Q21" t="str">
+      <c r="P21" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q21">
+        <v>31</v>
+      </c>
+      <c r="R21" t="str">
+        <v/>
+      </c>
+      <c r="S21">
+        <v>0.4</v>
+      </c>
+      <c r="T21" t="str">
         <v>Banten - Cilegon</v>
       </c>
-      <c r="R21" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S21" t="str">
-        <v>Suplai konsumen KTT MTSUI Kapasitas 31 MVA.</v>
-      </c>
-      <c r="T21" t="str">
-        <v/>
-      </c>
       <c r="U21" t="str">
-        <v/>
+        <v>JBB</v>
       </c>
       <c r="V21" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="str">
-        <v/>
-      </c>
-      <c r="C22" t="str">
-        <v>Feeder CLBRU ke KSTEL (Rencana)</v>
-      </c>
-      <c r="D22" t="str">
-        <v>PHT</v>
-      </c>
-      <c r="E22" t="str">
-        <v>CLBRU</v>
-      </c>
-      <c r="F22">
-        <v>1</v>
-      </c>
-      <c r="G22" t="str">
-        <v>KSTEL</v>
-      </c>
-      <c r="H22">
-        <v>3</v>
-      </c>
-      <c r="I22" t="str">
-        <v>150 kV</v>
-      </c>
-      <c r="J22">
-        <v>1</v>
-      </c>
-      <c r="K22">
-        <v>1</v>
-      </c>
-      <c r="L22" t="str">
-        <v>Beroperasi</v>
-      </c>
-      <c r="M22" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N22">
-        <v>50</v>
-      </c>
-      <c r="O22" t="str">
-        <v/>
-      </c>
-      <c r="P22">
-        <v>3.5</v>
-      </c>
-      <c r="Q22" t="str">
-        <v>Banten - Cilegon</v>
-      </c>
-      <c r="R22" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S22" t="str">
-        <v>Bay Rencana Penghantar KSTEL (Dashed Line).</v>
-      </c>
-      <c r="T22" t="str">
-        <v/>
-      </c>
-      <c r="U22" t="str">
-        <v/>
-      </c>
-      <c r="V22" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="str">
-        <v/>
-      </c>
-      <c r="C23" t="str">
-        <v>Feeder CLBRU ke POSCO (Rencana)</v>
-      </c>
-      <c r="D23" t="str">
-        <v>PHT</v>
-      </c>
-      <c r="E23" t="str">
-        <v>CLBRU</v>
-      </c>
-      <c r="F23">
-        <v>1</v>
-      </c>
-      <c r="G23" t="str">
-        <v>POSCO</v>
-      </c>
-      <c r="H23">
-        <v>3</v>
-      </c>
-      <c r="I23" t="str">
-        <v>150 kV</v>
-      </c>
-      <c r="J23">
-        <v>1</v>
-      </c>
-      <c r="K23">
-        <v>1</v>
-      </c>
-      <c r="L23" t="str">
-        <v>Beroperasi</v>
-      </c>
-      <c r="M23" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N23">
-        <v>50</v>
-      </c>
-      <c r="O23" t="str">
-        <v/>
-      </c>
-      <c r="P23">
-        <v>4.2</v>
-      </c>
-      <c r="Q23" t="str">
-        <v>Banten - Cilegon</v>
-      </c>
-      <c r="R23" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S23" t="str">
-        <v>Bay Rencana Penghantar POSCO (Dashed Line).</v>
-      </c>
-      <c r="T23" t="str">
-        <v/>
-      </c>
-      <c r="U23" t="str">
-        <v/>
-      </c>
-      <c r="V23" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" t="str">
-        <v/>
-      </c>
-      <c r="C24" t="str">
-        <v>Feeder CLGON ke KSTEL (Rencana)</v>
-      </c>
-      <c r="D24" t="str">
-        <v>PHT</v>
-      </c>
-      <c r="E24" t="str">
-        <v>CLGON</v>
-      </c>
-      <c r="F24">
-        <v>2</v>
-      </c>
-      <c r="G24" t="str">
-        <v>KSTEL-CLGON</v>
-      </c>
-      <c r="H24">
-        <v>3</v>
-      </c>
-      <c r="I24" t="str">
-        <v>150 kV</v>
-      </c>
-      <c r="J24">
-        <v>1</v>
-      </c>
-      <c r="K24">
-        <v>1</v>
-      </c>
-      <c r="L24" t="str">
-        <v>Beroperasi</v>
-      </c>
-      <c r="M24" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="N24">
-        <v>50</v>
-      </c>
-      <c r="O24" t="str">
-        <v/>
-      </c>
-      <c r="P24">
-        <v>2.8</v>
-      </c>
-      <c r="Q24" t="str">
-        <v>Banten - Cilegon</v>
-      </c>
-      <c r="R24" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="S24" t="str">
-        <v>Bay Rencana Penghantar KSTEL dari CLGON (Dashed Line).</v>
-      </c>
-      <c r="T24" t="str">
-        <v/>
-      </c>
-      <c r="U24" t="str">
-        <v/>
-      </c>
-      <c r="V24" t="str">
+        <v>Feeder Konsumen Industri KTT Mitsui</v>
+      </c>
+      <c r="W21" t="str">
+        <v/>
+      </c>
+      <c r="X21" t="str">
+        <v/>
+      </c>
+      <c r="Y21" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2152,7 +2133,7 @@
         <v>JBB</v>
       </c>
       <c r="N2" t="str">
-        <v/>
+        <v>Busbar 500 kV Suralaya Baru</v>
       </c>
       <c r="O2" t="str">
         <v/>
@@ -2205,7 +2186,7 @@
         <v>JBB</v>
       </c>
       <c r="N3" t="str">
-        <v/>
+        <v>Busbar 500 kV Suralaya</v>
       </c>
       <c r="O3" t="str">
         <v/>
@@ -2258,7 +2239,7 @@
         <v>JBB</v>
       </c>
       <c r="N4" t="str">
-        <v/>
+        <v>Busbar 500 kV Cilegon Baru</v>
       </c>
       <c r="O4" t="str">
         <v/>
@@ -2281,7 +2262,7 @@
         <v>Unit 3</v>
       </c>
       <c r="D5" t="str">
-        <v>Generator</v>
+        <v>Pembangkit</v>
       </c>
       <c r="E5" t="str">
         <v>Normal</v>
@@ -2311,7 +2292,7 @@
         <v>JBB</v>
       </c>
       <c r="N5" t="str">
-        <v>Bay Pembangkit: 1. Pembangkit, 2. Trafo Step-Up, 3. CB</v>
+        <v>Bay Pembangkit: 1. Pembangkit, 2. Trafo Generator, 3. CB</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -2417,16 +2398,16 @@
         <v>JBB</v>
       </c>
       <c r="N7" t="str">
-        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama.</v>
+        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #1,2 Suralaya 250 MVA).</v>
       </c>
       <c r="O7" t="str">
-        <v>Kondisi N-1-1 berdampak overload pada IBT Suralaya.</v>
+        <v>Overload pada IBT Suralaya.</v>
       </c>
       <c r="P7" t="str">
         <v>Terpasang DS OLS IBT 1,2 Suralaya.</v>
       </c>
       <c r="Q7" t="str">
-        <v>Uprating IBT–1 &amp; 2 menjadi 500 MVA.</v>
+        <v>Uprating IBT–1 &amp; 2 dari 250 MVA menjadi 500 MVA.</v>
       </c>
     </row>
     <row r="8">
@@ -2470,16 +2451,16 @@
         <v>JBB</v>
       </c>
       <c r="N8" t="str">
-        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama.</v>
+        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #4 Cilegon 500 MVA).</v>
       </c>
       <c r="O8" t="str">
-        <v>Overload saat gangguan kontinjensi.</v>
+        <v>Ketidakseimbangan beban.</v>
       </c>
       <c r="P8" t="str">
-        <v>Optimalisasi transfer trip dan defense scheme.</v>
+        <v>Optimalisasi transfer trip antar GI.</v>
       </c>
       <c r="Q8" t="str">
-        <v>Uprating IBT Suralaya.</v>
+        <v>Uprating IBT–1 &amp; 2 Suralaya menjadi 500 MVA.</v>
       </c>
     </row>
     <row r="9">
@@ -2487,16 +2468,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>Gardu Induk SRLYA (150 kV)</v>
+        <v>GI Suralaya 150 kV (Rel Busbar)</v>
       </c>
       <c r="C9" t="str">
         <v>SRLYA</v>
       </c>
       <c r="D9" t="str">
-        <v>Wide Busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="E9" t="str">
-        <v>Wide (Panjang)</v>
+        <v>Panjang (Wide Busbar)</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -2523,7 +2504,7 @@
         <v>JBB</v>
       </c>
       <c r="N9" t="str">
-        <v>Busbar 150 kV Suralaya (Membentang panjang menghubungkan Unit 3, IBT 2, IBT 1 ke SLRDA, PENDO, PENI, MCCI5)</v>
+        <v>Busbar 150 kV Suralaya (Menghubungkan IBT 1, IBT 2, dan Saluran Distribusi)</v>
       </c>
       <c r="O9" t="str">
         <v/>
@@ -2540,16 +2521,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>Gardu Induk CLBRU (150 kV)</v>
+        <v>GI Cilegon Baru 150 kV (Rel Busbar)</v>
       </c>
       <c r="C10" t="str">
         <v>CLBRU</v>
       </c>
       <c r="D10" t="str">
-        <v>Wide Busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="E10" t="str">
-        <v>Wide (Panjang)</v>
+        <v>Panjang (Wide Busbar)</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -2576,7 +2557,7 @@
         <v>JBB</v>
       </c>
       <c r="N10" t="str">
-        <v>Busbar 150 kV Cilegon Baru (Membentang menghubungkan IBT 4 ke CLGON, KSTEL, POSCO)</v>
+        <v>Busbar 150 kV Cilegon Baru</v>
       </c>
       <c r="O10" t="str">
         <v/>
@@ -2593,7 +2574,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>Gardu Induk SLRDA (150 kV)</v>
+        <v>GI Salira Indah</v>
       </c>
       <c r="C11" t="str">
         <v>SLRDA</v>
@@ -2629,7 +2610,7 @@
         <v>JBB</v>
       </c>
       <c r="N11" t="str">
-        <v>Busbar 150 kV Salira Indah</v>
+        <v>Gardu Induk Salira Indah</v>
       </c>
       <c r="O11" t="str">
         <v/>
@@ -2646,7 +2627,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>Gardu Induk PENDO (150 kV)</v>
+        <v>GI Pendo</v>
       </c>
       <c r="C12" t="str">
         <v>PENDO</v>
@@ -2682,7 +2663,7 @@
         <v>JBB</v>
       </c>
       <c r="N12" t="str">
-        <v>Busbar 150 kV Pendo</v>
+        <v>Gardu Induk Pendo</v>
       </c>
       <c r="O12" t="str">
         <v/>
@@ -2699,7 +2680,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>Gardu Induk PENI (150 kV)</v>
+        <v>GI Chandra Asri (PENI)</v>
       </c>
       <c r="C13" t="str">
         <v>PENI</v>
@@ -2735,16 +2716,16 @@
         <v>JBB</v>
       </c>
       <c r="N13" t="str">
-        <v>Ruas Penghantar Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
+        <v>Ruas Penghantar Suralaya-PENI masih single phi.</v>
       </c>
       <c r="O13" t="str">
-        <v>Pemadaman apabila terjadi gangguan N-1-1.</v>
+        <v>Pemadaman apabila terdapat gangguan N-1-1.</v>
       </c>
       <c r="P13" t="str">
-        <v>Penyesuaian jadwal pemeliharaan dari KTT.</v>
+        <v>Pemeliharaan mengikuti jadwal KTT.</v>
       </c>
       <c r="Q13" t="str">
-        <v>Usulan Double phi.</v>
+        <v>Double phi COD 2030.</v>
       </c>
     </row>
     <row r="14">
@@ -2752,7 +2733,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>Gardu Induk MCCI5 (150 kV)</v>
+        <v>GI Mitsubishi Chemical (MCCI)</v>
       </c>
       <c r="C14" t="str">
         <v>MCCI5</v>
@@ -2788,16 +2769,16 @@
         <v>JBB</v>
       </c>
       <c r="N14" t="str">
-        <v>Ruas Penghantar Suralaya–MCCI–Cilegon masih single phi.</v>
+        <v>Ruas Penghantar Suralaya-MCCI-Cilegon masih single phi.</v>
       </c>
       <c r="O14" t="str">
-        <v>Pemeliharaan penghantar sulit dilakukan.</v>
+        <v>Pemadaman apabila gangguan.</v>
       </c>
       <c r="P14" t="str">
-        <v>Pengaturan konfigurasi jaringan.</v>
+        <v>Penyesuaian jadwal pemeliharaan.</v>
       </c>
       <c r="Q14" t="str">
-        <v>Usulan Double phi.</v>
+        <v>Usulan double phi ruas Suralaya s.d Cilegon Lama.</v>
       </c>
     </row>
     <row r="15">
@@ -2805,7 +2786,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>Gardu Induk CLGON (150 kV)</v>
+        <v>GI Cilegon Lama</v>
       </c>
       <c r="C15" t="str">
         <v>CLGON</v>
@@ -2841,7 +2822,7 @@
         <v>JBB</v>
       </c>
       <c r="N15" t="str">
-        <v>Busbar 150 kV Cilegon Lama (Menerima 2 Line dari CLBRU)</v>
+        <v>Gardu Induk Cilegon Lama</v>
       </c>
       <c r="O15" t="str">
         <v/>
@@ -2858,7 +2839,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>Gardu Induk MTSUI (150 kV)</v>
+        <v>GI Mitsui (MTSUI)</v>
       </c>
       <c r="C16" t="str">
         <v>MTSUI</v>
@@ -2894,16 +2875,16 @@
         <v>JBB</v>
       </c>
       <c r="N16" t="str">
-        <v>Ruas Peni–Mitsui–Cilegon masih single phi.</v>
+        <v>Ruas Mitsui-Cilegon single phi</v>
       </c>
       <c r="O16" t="str">
-        <v>Pemadaman apabila trip saat pembebanan tinggi.</v>
+        <v/>
       </c>
       <c r="P16" t="str">
-        <v>Pengaturan konfigurasi jaringan.</v>
+        <v/>
       </c>
       <c r="Q16" t="str">
-        <v>Usulan Double phi.</v>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -3094,10 +3075,10 @@
         <v/>
       </c>
       <c r="J20" t="str">
-        <v>Normal</v>
+        <v>N-1</v>
       </c>
       <c r="K20" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="L20" t="str">
         <v>Banten</v>
@@ -3106,7 +3087,7 @@
         <v>JBB</v>
       </c>
       <c r="N20" t="str">
-        <v>Konsumen Tegangan Tinggi PENI</v>
+        <v>Konsumen Tegangan Tinggi PENI Chandra Asri</v>
       </c>
       <c r="O20" t="str">
         <v/>
@@ -3159,7 +3140,7 @@
         <v>JBB</v>
       </c>
       <c r="N21" t="str">
-        <v>Konsumen Tegangan Tinggi LCI (Dipasok 2 Sirkit)</v>
+        <v>Konsumen KTT LCI</v>
       </c>
       <c r="O21" t="str">
         <v/>
@@ -3212,7 +3193,7 @@
         <v>JBB</v>
       </c>
       <c r="N22" t="str">
-        <v>Konsumen Tegangan Tinggi MCCI</v>
+        <v>Konsumen KTT MCCI</v>
       </c>
       <c r="O22" t="str">
         <v/>
@@ -3265,7 +3246,7 @@
         <v>JBB</v>
       </c>
       <c r="N23" t="str">
-        <v>Konsumen Tegangan Tinggi MTSUI</v>
+        <v>Konsumen KTT Mitsui</v>
       </c>
       <c r="O23" t="str">
         <v/>
@@ -3286,7 +3267,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3307,70 +3288,70 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Peralatan (5)</v>
+        <v>Peralatan (1)</v>
       </c>
       <c r="B2" t="str">
-        <v>Busbar</v>
+        <v>Generator / Pembangkit</v>
       </c>
       <c r="C2" t="str">
-        <v>Batang Rel Horizontal Tebal (Cyan/Biru)</v>
+        <v>Lingkaran Hijau dengan Gelombang Sinus AC (~)</v>
       </c>
       <c r="D2" t="str">
-        <v>Batang konduktor utama di Gardu Induk (GI / GITET) yang mengumpulkan dan membagikan daya listrik.</v>
+        <v>Titik hulu pembangkit listrik utama (PLTU, PLTA, PLTG, PLTGU).</v>
       </c>
       <c r="E2" t="str">
-        <v>Suralaya Baru (500 kV), GI SLRDA (150 kV)</v>
+        <v>PLTU Suralaya Unit 3 (600 MW)</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Peralatan (5)</v>
+        <v>Peralatan (2)</v>
       </c>
       <c r="B3" t="str">
-        <v>Wide Busbar</v>
+        <v>Trafo Generator (GSUT)</v>
       </c>
       <c r="C3" t="str">
-        <v>Batang Rel Horizontal Panjang Membentang</v>
+        <v>2 Lingkaran Interlocking (Atas: Hijau sisi Gen, Bawah: Merah sisi GI)</v>
       </c>
       <c r="D3" t="str">
-        <v>Batang rel busbar panjang untuk GI hub yang terhubung ke 3 atau lebih GI/feeder agar jalur transmisi tidak semrawut.</v>
+        <v>Trafo penaik tegangan generator (Generator Step-Up) dari 15-20 kV ke tegangan tinggi GI (150/500 kV).</v>
       </c>
       <c r="E3" t="str">
-        <v>SRLYA (150 kV), CLBRU (150 kV)</v>
+        <v>Bay Pembangkit ke Busbar GI</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Peralatan (5)</v>
+        <v>Switching (3)</v>
       </c>
       <c r="B4" t="str">
-        <v>Generator</v>
+        <v>CB / PMT (Pemutus Tenaga)</v>
       </c>
       <c r="C4" t="str">
-        <v>Lingkaran Hijau dengan Gelombang AC (~) &amp; Terminal Bulatan</v>
+        <v>Balok / Persegi Panjang Solid Merah Tegak dengan garis terminal</v>
       </c>
       <c r="D4" t="str">
-        <v>Unit pembangkit tenaga listrik (PLTU, PLTA, PLTGU) lengkap dengan bay PMT dan trafo penaik tegangan.</v>
+        <v>Circuit Breaker pada bay pengirim dan penerima GI ke GI untuk memutus beban dan gangguan arus pendek.</v>
       </c>
       <c r="E4" t="str">
-        <v>PLTU Suralaya Unit 3 (600 MW)</v>
+        <v>Bay Line, Bay IBT, Bay Trafo, Bay Generator</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Peralatan (5)</v>
+        <v>Peralatan (4)</v>
       </c>
       <c r="B5" t="str">
-        <v>IBT</v>
+        <v>IBT (Interbus Transformer)</v>
       </c>
       <c r="C5" t="str">
-        <v>3 Lingkaran Interlocking (Biru, Merah, Kuning) + Badge Nomor</v>
+        <v>3 Lingkaran Bertumpuk (Atas Biru 500kV, Kiri Merah 150kV, Kanan Kuning 33kV)</v>
       </c>
       <c r="D5" t="str">
-        <v>Inter-bus Transformer tegangan ekstra tinggi (500/150 kV atau 275/150 kV) dengan 3 belitan (primer, sekunder, tersier).</v>
+        <v>Trafo interkoneksi sistem transmisi tegangan ekstra tinggi (500/150 kV atau 275/150 kV).</v>
       </c>
       <c r="E5" t="str">
-        <v>IBT 1 Suralaya (250 MVA), IBT 4 Cilegon Baru (500 MVA)</v>
+        <v>IBT 1 &amp; 2 Suralaya (250 MVA), IBT 4 Cilegon (500 MVA)</v>
       </c>
     </row>
     <row r="6">
@@ -3378,106 +3359,72 @@
         <v>Peralatan (5)</v>
       </c>
       <c r="B6" t="str">
-        <v>Trafo</v>
+        <v>Trafo Distribusi</v>
       </c>
       <c r="C6" t="str">
-        <v>2 Lingkaran Interlocking (Merah &amp; Hijau) + Terminal Bulatan</v>
+        <v>2 Lingkaran Interlocking (Atas: Merah 150kV, Bawah: Kuning 20kV / 70kV)</v>
       </c>
       <c r="D6" t="str">
-        <v>Trafo penurun tegangan (Step-down / Distribusi) 150/20 kV untuk menyuplai penyulang beban lokal.</v>
+        <v>Trafo step-down daya di Gardu Induk yang menurunkan tegangan dari 150 kV ke 70 kV atau 20 kV.</v>
       </c>
       <c r="E6" t="str">
-        <v>Trafo Distribusi 150/20 kV GI Salira Indah</v>
+        <v>Trafo 150/20 kV GI Distribusi / Feeder KTT</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Peralatan (5)</v>
+        <v>Peralatan (6)</v>
       </c>
       <c r="B7" t="str">
-        <v>Beban</v>
+        <v>Busbar</v>
       </c>
       <c r="C7" t="str">
-        <v>Segitiga Terbalik (∇) dengan Terminal Bulatan di Atas</v>
+        <v>Batang Rel Horizontal Tebal (Cyan/Biru)</v>
       </c>
       <c r="D7" t="str">
-        <v>Konsumen Tegangan Tinggi (KTT industri), penyulang distribusi, atau titik beban pemakaian tenaga listrik.</v>
+        <v>Batang konduktor utama di Gardu Induk (GI / GITET) yang mengumpulkan dan membagikan daya listrik.</v>
       </c>
       <c r="E7" t="str">
-        <v>KTT SLFDO-1 (78 MVA), KTT LCI (115 MVA), KTT MCCI</v>
+        <v>Suralaya Baru (500 kV), GI SRLYA 150 kV, GI CLBRU 150 kV</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Peralatan (5)</v>
+        <v>Peralatan (7)</v>
       </c>
       <c r="B8" t="str">
-        <v>PHT</v>
+        <v>Beban</v>
       </c>
       <c r="C8" t="str">
-        <v>Garis Kapsul Transmisi dengan 2 Bulatan di Kedua Ujung</v>
+        <v>Segitiga Terbalik (∇) Kuning Emas dengan terminal bulatan di atas</v>
       </c>
       <c r="D8" t="str">
-        <v>Penghantar Transmisi Saluran Udara (SUTET 500 kV / SUTT 150 kV) atau Saluran Kabel Bawah Tanah (SKTT).</v>
+        <v>Simbol resmi beban listrik konsumen industri KTT (Konsumen Tegangan Tinggi) atau feeder beban.</v>
       </c>
       <c r="E8" t="str">
-        <v>SUTT 150 kV SRLYA - PENI, SUTET 500 kV Tambun - Cawang</v>
+        <v>KTT SLFDO-1 (78 MVA), KTT PENI (40 MVA), KTT LCI (115 MVA)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Switching (2)</v>
+        <v>Peralatan (8)</v>
       </c>
       <c r="B9" t="str">
-        <v>PMT (Circuit Breaker)</v>
+        <v>PHT (Penghantar)</v>
       </c>
       <c r="C9" t="str">
-        <v>Sakelar Kontak Terbuka dengan Tanda Silang (X)</v>
+        <v>Kapsul Saluran Transmisi dengan dua bulatan terminal di ujung</v>
       </c>
       <c r="D9" t="str">
-        <v>Pemutus Tenaga: peralatan sakelar yang mampu membuka dan menutup sirkit dalam kondisi normal maupun kondisi hubung singkat (gangguan).</v>
+        <v>Saluran udara/kabel transmisi tenaga listrik penghubung antar gardu induk.</v>
       </c>
       <c r="E9" t="str">
-        <v>PMT Bay Pembangkit, PMT Bay IBT, PMT Bay Penghantar</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Switching (2)</v>
-      </c>
-      <c r="B10" t="str">
-        <v>PMS (Disconnector)</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Sakelar Pemisah dengan Garis Huruf (T)</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Pemisah: peralatan sakelar mekanis untuk memisahkan bagian instalasi yang bertegangan dari yang tidak bertegangan saat kondisi tanpa beban untuk keselamatan kerja.</v>
-      </c>
-      <c r="E10" t="str">
-        <v>PMS Busbar, PMS Line, PMS Tanah</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Penghubung (1)</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Connection Node</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Lingkaran Bulat Koneksi / Junction Point</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Titik simpul percabangan saluran listrik atau tap-off feeder.</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Junction busbar tap, simpul interkoneksi</v>
+        <v>PHT Suralaya - Salira Indah, PHT Suralaya - PENI</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3564,8 +3511,8 @@
 2. Kondisi N–1–1 (IBT Suralaya dan IBT Cilegon) berdampak overload pada IBT Suralaya yang beroperasi.</v>
       </c>
       <c r="G3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW.
-2. Rencana penambahan target DS OLS SS Suralaya 1,2.
+        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW (Berdasarkan buku DS Tahun 2025).
+2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan total target sebesar 137 MW (Berdasarkan buku DS Tahun 2025).
 3. Pemeliharaan IBT saat beban rendah dan pada saat PLTU Suralaya Unit–3 beroperasi.</v>
       </c>
       <c r="H3" t="str" xml:space="preserve">

</xml_diff>